<commit_message>
MODELLING - sentiment_atribution.py dejo intento final de to_customer_needs(). Todavia pueden cambiar palabras relacionadas o valores de algunos parametros create_relation_matrix --> borra atrib o cust needs sin relacion
DATA PREPARATION
- clean_data.py. Desarrolle funcion drop_alternatives_with_wrong_values.
- construct_data.py. Mejore identificacion de customer needs. Flexibilice parametros
</commit_message>
<xml_diff>
--- a/data/data_preparation/customer_needs_celulares.xlsx
+++ b/data/data_preparation/customer_needs_celulares.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,7 +469,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>tiene buen sonido</t>
+          <t>tiene buena señal</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>buena capacidad memoria</t>
+          <t>tiene buen sonido</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>buena pantalla buena</t>
+          <t>buena capacidad memoria</t>
         </is>
       </c>
     </row>
@@ -499,7 +499,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>tiene carga rapida</t>
+          <t>buena pantalla buena</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,107 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>tiene carga rapida</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>desbloqueo huella digital</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>corre bien juegos</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>trae cargador cable</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>tiene buen tamaño</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>varias aplicaciones abiertas</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>calidad fotos videos</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>sistema operativo rapido</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>bien procesador rapido</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>primera compro marca</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>celular lindo diseño</t>
         </is>
       </c>
     </row>

</xml_diff>